<commit_message>
Added New For Family and Community Use Land
</commit_message>
<xml_diff>
--- a/Land/New Microsoft Excel Worksheet.xlsx
+++ b/Land/New Microsoft Excel Worksheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anower H. Faysal\Desktop\Survival\Escape-Matrix-Hub-full-self-sufficiant\Land\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E4CA962-1EA3-4D89-A6F2-EE84266B5965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{826E25E1-1257-4D20-A4F4-57D85FFF5458}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Single Use" sheetId="2" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="52">
   <si>
     <t>Reason</t>
   </si>
@@ -63,14 +63,142 @@
   </si>
   <si>
     <t>House ( 1Bed + 1Bath + Kitchen + Stor. Space)</t>
+  </si>
+  <si>
+    <t>Water Zone ( Tube Well  + WP )</t>
+  </si>
+  <si>
+    <t>Biogas + Wood Storage</t>
+  </si>
+  <si>
+    <t>Medical herb</t>
+  </si>
+  <si>
+    <t>Fenching</t>
+  </si>
+  <si>
+    <t>Extra</t>
+  </si>
+  <si>
+    <t>Rice Field (Year Round)</t>
+  </si>
+  <si>
+    <t>Vegetable (Year Round)</t>
+  </si>
+  <si>
+    <t>Tree (Fruits)</t>
+  </si>
+  <si>
+    <t>Pond (Fish + Water + Duck)</t>
+  </si>
+  <si>
+    <t>Farm Room (Chicken + Rabbit + Goat + 1–2 Cow)</t>
+  </si>
+  <si>
+    <t>Water Zone (Tube Well + WP)</t>
+  </si>
+  <si>
+    <t>Medical Herb</t>
+  </si>
+  <si>
+    <t>Fencing</t>
+  </si>
+  <si>
+    <t>Extra / Buffer / Path</t>
+  </si>
+  <si>
+    <t>House 4P (3Bed + 2Bath + Kitchen + Storage)</t>
+  </si>
+  <si>
+    <t>Residential Area (50 family houses)</t>
+  </si>
+  <si>
+    <t>Rice Field</t>
+  </si>
+  <si>
+    <t>Vegetable Farming</t>
+  </si>
+  <si>
+    <t>Fruit Orchard</t>
+  </si>
+  <si>
+    <t>Spice Farming</t>
+  </si>
+  <si>
+    <t>Animal Feed Field</t>
+  </si>
+  <si>
+    <t>Cow &amp; Goat Farm</t>
+  </si>
+  <si>
+    <t>Chicken/Duck/Rabbit Area</t>
+  </si>
+  <si>
+    <t>Fish Pond + Water Reserve</t>
+  </si>
+  <si>
+    <t>Compost &amp; Waste Processing</t>
+  </si>
+  <si>
+    <t>Biogas Plant Area</t>
+  </si>
+  <si>
+    <t>Medical Herb Garden</t>
+  </si>
+  <si>
+    <t>Tube-well + Water Infrastructure</t>
+  </si>
+  <si>
+    <t>Food Storage / Grain Silos</t>
+  </si>
+  <si>
+    <t>Seed Bank &amp; Nursery</t>
+  </si>
+  <si>
+    <t>Solar / Energy Zone</t>
+  </si>
+  <si>
+    <t>Woodlot / Bamboo Forest</t>
+  </si>
+  <si>
+    <t>Community Kitchen + Bakery</t>
+  </si>
+  <si>
+    <t>Workshop / Repair Area</t>
+  </si>
+  <si>
+    <t>Clinic / Medical Center</t>
+  </si>
+  <si>
+    <t>School / Learning Center</t>
+  </si>
+  <si>
+    <t>Community Hall / Shelter</t>
+  </si>
+  <si>
+    <t>Road + Path + Drainage</t>
+  </si>
+  <si>
+    <t>Security Buffer + Fence</t>
+  </si>
+  <si>
+    <t>Emergency Extra Reserve</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -106,9 +234,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -389,7 +529,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7DA3D4E-1842-4858-A9F5-300AE71B5EB8}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.140625" customWidth="1"/>
@@ -445,7 +585,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -478,6 +618,46 @@
       </c>
       <c r="B10">
         <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -487,7 +667,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.85546875" customWidth="1"/>
@@ -506,6 +686,118 @@
         <v>2</v>
       </c>
     </row>
+    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="3">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -514,7 +806,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3365102D-D8A7-49FC-B002-9E879B5F37E0}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.28515625" customWidth="1"/>
@@ -523,14 +815,212 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="3">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="3">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="3">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="3">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="3">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="3">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="3">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="3">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="3">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" s="3">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="3">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="3">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" s="3">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B18" s="3">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" s="3">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="3">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B23" s="3">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B24" s="3">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B25" s="3">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" s="3">
+        <v>1500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added New For My Family
</commit_message>
<xml_diff>
--- a/Land/New Microsoft Excel Worksheet.xlsx
+++ b/Land/New Microsoft Excel Worksheet.xlsx
@@ -8,26 +8,38 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anower H. Faysal\Desktop\Survival\Escape-Matrix-Hub-full-self-sufficiant\Land\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{826E25E1-1257-4D20-A4F4-57D85FFF5458}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E5E8509-3829-470E-851F-9EA59BF5CDBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Single Use" sheetId="2" r:id="rId1"/>
     <sheet name="Family Use" sheetId="1" r:id="rId2"/>
     <sheet name="Community Use" sheetId="3" r:id="rId3"/>
+    <sheet name="My Family" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="67">
   <si>
     <t>Reason</t>
   </si>
@@ -183,6 +195,51 @@
   </si>
   <si>
     <t>Emergency Extra Reserve</t>
+  </si>
+  <si>
+    <t>Vegetable Farming (Year Round)</t>
+  </si>
+  <si>
+    <t>Survival Crops (Potato + Sweet Potato + Cassava + Pumpkin)</t>
+  </si>
+  <si>
+    <t>Compost + Vermicompost Area</t>
+  </si>
+  <si>
+    <t>Farm Area (Chicken + Rabbit + Goat + 2 Cow)</t>
+  </si>
+  <si>
+    <t>Animal Feed Field (Grass + Fodder Trees)</t>
+  </si>
+  <si>
+    <t>Bamboo / Woodlot Area</t>
+  </si>
+  <si>
+    <t>Water Zone (Tube Well + Water Pump + Wash Area)</t>
+  </si>
+  <si>
+    <t>Food Storage / Dry Storage / Grain Storage</t>
+  </si>
+  <si>
+    <t>Seed Bank + Nursery</t>
+  </si>
+  <si>
+    <t>Solar + Utility Zone</t>
+  </si>
+  <si>
+    <t>Path + Drainage + Working Space</t>
+  </si>
+  <si>
+    <t>Fencing + Security Buffer</t>
+  </si>
+  <si>
+    <t>Extra Emergency Reserve Land</t>
+  </si>
+  <si>
+    <t>House (4Bed + 3Bath + Kitchen + Storage + Utility</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
 </sst>
 </file>
@@ -1026,4 +1083,195 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EC75069-8ED3-4D31-A354-6B6D8A847A49}">
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="52.42578125" customWidth="1"/>
+    <col min="2" max="2" width="37.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2" s="5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="5">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="5">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="5">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="5">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="5">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" s="5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B12" s="5">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" s="5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B18" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B19" s="5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B20" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B21" s="5">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>66</v>
+      </c>
+      <c r="B26">
+        <f>SUM(B2:B21)</f>
+        <v>479</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>